<commit_message>
butter filter and strategy 2
</commit_message>
<xml_diff>
--- a/results_v3.xlsx
+++ b/results_v3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="454" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-10000" yWindow="-21710" windowWidth="38620" windowHeight="21100" tabRatio="454" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,9 +16,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -80,35 +87,36 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -400,28 +408,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:AT62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.21875" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="15.44140625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="15.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="23.6640625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="19.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="14.109375" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="13.88671875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="14.109375" bestFit="1" customWidth="1" style="11" min="9" max="9"/>
-    <col width="33.5546875" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="14.44140625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="13.88671875" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="15.21875" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="14.6640625" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="12" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="15.44140625" customWidth="1" min="4" max="4"/>
+    <col width="15.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="23.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="23" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="19.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="14.109375" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="14.109375" customWidth="1" min="10" max="10"/>
+    <col width="13.88671875" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="14.109375" bestFit="1" customWidth="1" style="11" min="12" max="12"/>
+    <col width="33.5546875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="14.44140625" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="13.88671875" bestFit="1" customWidth="1" min="15" max="15"/>
     <col width="15.21875" bestFit="1" customWidth="1" min="16" max="16"/>
     <col width="14.6640625" bestFit="1" customWidth="1" min="17" max="17"/>
     <col width="12" bestFit="1" customWidth="1" min="18" max="18"/>
     <col width="15.21875" bestFit="1" customWidth="1" min="19" max="19"/>
     <col width="14.6640625" bestFit="1" customWidth="1" min="20" max="20"/>
+    <col width="12" bestFit="1" customWidth="1" min="21" max="21"/>
+    <col width="15.21875" bestFit="1" customWidth="1" min="22" max="22"/>
+    <col width="14.6640625" bestFit="1" customWidth="1" min="23" max="23"/>
+    <col width="16.77734375" bestFit="1" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="8">
@@ -442,92 +454,217 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>delta_t_empiric</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>delta_G_formula</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>delta_G_PV_personalized</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>delta_t_PV_personalized</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>FIT_PV_personalized</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>delta_G_101</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>delta_t_101</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>FIT_101</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>delta_G_101</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>FIT_SSM_34</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>delta_G_SSM_34</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>FIT_SSM_35</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>delta_G_SSM_35</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>delta_t_SSM_35</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>FIT_SSM_38</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>delta_G_SSM_38</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>delta_t_SSM_38</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>FIT_SSM_39</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>delta_G_SSM_39</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" s="13" t="inlineStr">
         <is>
           <t>delta_t_SSM_39</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>delta_t_SSM_34</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_s2_34_s2</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_s2_34</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_s2_34</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_s2_34</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_44</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_44</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_44</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_45</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_45</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_45</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_46</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_46</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_46</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_54</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_54</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_54</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_64</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_64</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_64</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>FIT_SSM_74</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>delta_G_SSM_74</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>delta_t_SSM_74</t>
         </is>
       </c>
     </row>
@@ -555,33 +692,69 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>21.75627697275417</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="n">
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="n">
         <v>-76.7218</v>
       </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>69.08353269100189</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>66.20668023824692</v>
       </c>
-      <c r="O2" t="n">
+      <c r="R2" t="n">
         <v>79.75425720214844</v>
       </c>
-      <c r="R2" t="n">
+      <c r="U2" t="n">
         <v>70.09125947952271</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>16.28593504428864</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>69.47198361158371</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>65.92199802398682</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>66.53335839509964</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>64.83224034309387</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>70.00838667154312</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>68.24367046356201</v>
       </c>
     </row>
     <row r="3">
@@ -608,33 +781,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>9.846218852866473</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="n">
         <v>-372.8777</v>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>52.06067115068436</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>45.20611464977264</v>
       </c>
-      <c r="O3" t="n">
+      <c r="R3" t="n">
         <v>77.99473479390144</v>
       </c>
-      <c r="R3" t="n">
+      <c r="U3" t="n">
         <v>60.0797176361084</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>57.57713615894318</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>56.43520653247833</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>55.28586059808731</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>55.04221022129059</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>59.63287502527237</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>59.66007262468338</v>
       </c>
     </row>
     <row r="4">
@@ -661,33 +867,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>-4.242890543785793</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="n">
         <v>-343.5359</v>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
         <v>51.62617564201355</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>56.28854930400848</v>
       </c>
-      <c r="O4" t="n">
+      <c r="R4" t="n">
         <v>77.20123007893562</v>
       </c>
-      <c r="R4" t="n">
+      <c r="U4" t="n">
         <v>54.95941638946533</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>60.34316420555115</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>49.7981995344162</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>51.67513191699982</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>50.06779432296753</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>62.25874722003937</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>59.11823958158493</v>
       </c>
     </row>
     <row r="5">
@@ -714,33 +953,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>-11.32878279993903</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="n">
         <v>-609.2437</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
         <v>42.16179251670837</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>39.0783816576004</v>
       </c>
-      <c r="O5" t="n">
+      <c r="R5" t="n">
         <v>78.7266843020916</v>
       </c>
-      <c r="R5" t="n">
+      <c r="U5" t="n">
         <v>45.93673050403595</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>46.87333703041077</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>42.20720231533051</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>41.57096445560455</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>41.90168976783752</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>42.45462119579315</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>52.04640775918961</v>
       </c>
     </row>
     <row r="6">
@@ -767,33 +1039,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>-13.39650663638063</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n">
         <v>-74.2556</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
         <v>66.3923367857933</v>
       </c>
-      <c r="L6" t="n">
+      <c r="O6" t="n">
         <v>64.47644233703613</v>
       </c>
-      <c r="O6" t="n">
+      <c r="R6" t="n">
         <v>76.11759305000305</v>
       </c>
-      <c r="R6" t="n">
+      <c r="U6" t="n">
         <v>66.84568822383881</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>65.34521281719208</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>64.80675339698792</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>60.7750877737999</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>66.05682969093323</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>66.58786982297897</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>67.56705343723297</v>
       </c>
     </row>
     <row r="7">
@@ -820,33 +1125,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>52.23483111059972</v>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="n">
         <v>12.773</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
         <v>67.2761082649231</v>
       </c>
-      <c r="L7" t="n">
+      <c r="O7" t="n">
         <v>67.04623699188232</v>
       </c>
-      <c r="O7" t="n">
+      <c r="R7" t="n">
         <v>81.32179901003838</v>
       </c>
-      <c r="R7" t="n">
+      <c r="U7" t="n">
         <v>68.18967312574387</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>68.07649433612823</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>67.26454794406891</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>67.30702370405197</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>62.57957816123962</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>71.32580578327179</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>70.85898965597153</v>
       </c>
     </row>
     <row r="8">
@@ -873,30 +1211,63 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>21.53590739539882</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="n">
         <v>-54.1804</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
         <v>66.37006998062134</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="n">
         <v>66.68574512004852</v>
       </c>
-      <c r="O8" t="n">
+      <c r="R8" t="n">
         <v>81.20083510875702</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>68.71384829282761</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>67.53817200660706</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>67.79297590255737</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>67.80176311731339</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>68.5833066701889</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>72.30484038591385</v>
       </c>
     </row>
     <row r="9">
@@ -923,33 +1294,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>44.22402232364951</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="n">
         <v>-73.1135</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
         <v>71.90750241279602</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="n">
         <v>71.82801812887192</v>
       </c>
-      <c r="O9" t="n">
+      <c r="R9" t="n">
         <v>78.4210316836834</v>
       </c>
-      <c r="R9" t="n">
+      <c r="U9" t="n">
         <v>72.04775959253311</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>72.3018079996109</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>70.9658682346344</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>71.27694636583328</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>71.89353108406067</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>72.03119546175003</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>75.48670694231987</v>
       </c>
     </row>
     <row r="10">
@@ -976,33 +1380,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>3.367201685442034</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="n">
         <v>-31.6868</v>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
         <v>70.63945680856705</v>
       </c>
-      <c r="L10" t="n">
+      <c r="O10" t="n">
         <v>69.54242438077927</v>
       </c>
-      <c r="O10" t="n">
+      <c r="R10" t="n">
         <v>81.80320709943771</v>
       </c>
-      <c r="R10" t="n">
+      <c r="U10" t="n">
         <v>71.34441435337067</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>69.29309368133545</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>69.88862603902817</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>70.75566947460175</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>68.1087926030159</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>73.13592284917831</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>74.83513876795769</v>
       </c>
     </row>
     <row r="11">
@@ -1029,33 +1466,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>53.62774720314039</v>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="n">
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>-167.9497</v>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
         <v>55.88486790657043</v>
       </c>
-      <c r="L11" t="n">
+      <c r="O11" t="n">
         <v>57.54047036170959</v>
       </c>
-      <c r="O11" t="n">
+      <c r="R11" t="n">
         <v>77.78621092438698</v>
       </c>
-      <c r="R11" t="n">
+      <c r="U11" t="n">
         <v>60.14551669359207</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>61.61510050296783</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>51.8587738275528</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>57.59016871452332</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>57.50561207532883</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>64.34017419815063</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>63.7894794344902</v>
       </c>
     </row>
     <row r="12">
@@ -1082,33 +1552,69 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>25.61241932041938</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="n">
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="n">
         <v>-77.7002</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
         <v>66.06106162071228</v>
       </c>
-      <c r="L12" t="n">
+      <c r="O12" t="n">
         <v>56.76135122776031</v>
       </c>
-      <c r="O12" t="n">
+      <c r="R12" t="n">
         <v>70.54352462291718</v>
       </c>
-      <c r="R12" t="n">
+      <c r="U12" t="n">
         <v>59.9481076002121</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>-6.41627311706543</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>64.36360776424408</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>58.24914872646332</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>59.95423495769501</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>57.10373818874359</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>56.12501800060272</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>61.16631627082825</v>
       </c>
     </row>
     <row r="13">
@@ -1135,33 +1641,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>10.0404121965947</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="n">
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="n">
         <v>-332.0777</v>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
         <v>46.11070156097412</v>
       </c>
-      <c r="L13" t="n">
+      <c r="O13" t="n">
         <v>43.73747110366821</v>
       </c>
-      <c r="O13" t="n">
+      <c r="R13" t="n">
         <v>78.29841822385788</v>
       </c>
-      <c r="R13" t="n">
+      <c r="U13" t="n">
         <v>52.89991497993469</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>51.42034888267517</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>46.41999006271362</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>46.68156504631042</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>47.05823063850403</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>48.40677976608276</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>55.14932870864868</v>
       </c>
     </row>
     <row r="14">
@@ -1188,33 +1727,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>-2.362629576594233</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="n">
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="n">
         <v>-362.8828</v>
       </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
         <v>46.62092328071594</v>
       </c>
-      <c r="L14" t="n">
+      <c r="O14" t="n">
         <v>51.67661905288696</v>
       </c>
-      <c r="O14" t="n">
+      <c r="R14" t="n">
         <v>71.62388563156128</v>
       </c>
-      <c r="R14" t="n">
+      <c r="U14" t="n">
         <v>51.70677006244659</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>55.52425980567932</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>47.57181406021118</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>46.4893639087677</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>47.58503437042236</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>50.71265995502472</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>57.36711621284485</v>
       </c>
     </row>
     <row r="15">
@@ -1241,33 +1813,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>-7.458485764161993</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="n">
         <v>-512.5972</v>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
         <v>24.53176975250244</v>
       </c>
-      <c r="L15" t="n">
+      <c r="O15" t="n">
         <v>29.2177140712738</v>
       </c>
-      <c r="O15" t="n">
+      <c r="R15" t="n">
         <v>73.42918813228607</v>
       </c>
-      <c r="R15" t="n">
+      <c r="U15" t="n">
         <v>31.16289377212524</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>30.08611798286438</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>25.06294846534729</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>24.34881329536438</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>24.21244382858276</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>30.7392954826355</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>43.26233267784119</v>
       </c>
     </row>
     <row r="16">
@@ -1294,34 +1899,67 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>-24.55571974484543</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="n">
         <v>-61.1459</v>
       </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
         <v>53.46926152706146</v>
       </c>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" t="n">
+      <c r="N16" s="10" t="n"/>
+      <c r="O16" t="n">
         <v>55.06239831447601</v>
       </c>
-      <c r="O16" t="n">
+      <c r="R16" t="n">
         <v>68.94195973873138</v>
       </c>
-      <c r="R16" t="n">
+      <c r="U16" t="n">
         <v>54.99742329120636</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>54.79158461093903</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>54.61820960044861</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>49.38650131225586</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>54.70118820667267</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>48.48794341087341</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>58.67908298969269</v>
       </c>
     </row>
     <row r="17">
@@ -1348,33 +1986,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>49.98437939359683</v>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="n">
         <v>8.423999999999999</v>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
         <v>66.91068410873413</v>
       </c>
-      <c r="L17" t="n">
+      <c r="O17" t="n">
         <v>65.96070826053619</v>
       </c>
-      <c r="O17" t="n">
+      <c r="R17" t="n">
         <v>78.31141501665115</v>
       </c>
-      <c r="R17" t="n">
+      <c r="U17" t="n">
         <v>67.50281155109406</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>68.10216307640076</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>66.56338274478912</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>67.42299497127533</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>61.42402291297913</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>69.65576112270355</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>71.08277678489685</v>
       </c>
     </row>
     <row r="18">
@@ -1401,30 +2072,63 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>17.00646420489879</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="n">
         <v>-57.6554</v>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
         <v>63.18274736404419</v>
       </c>
-      <c r="L18" t="n">
+      <c r="O18" t="n">
         <v>66.30968749523163</v>
       </c>
-      <c r="O18" t="n">
+      <c r="R18" t="n">
         <v>76.50259137153625</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>65.79295098781586</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>64.87802267074585</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>64.63422775268555</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>64.30277526378632</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>66.58384203910828</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>69.11877691745758</v>
       </c>
     </row>
     <row r="19">
@@ -1451,33 +2155,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>42.7518616717111</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="n">
         <v>-72.9786</v>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
         <v>70.5456018447876</v>
       </c>
-      <c r="L19" t="n">
+      <c r="O19" t="n">
         <v>66.03844165802002</v>
       </c>
-      <c r="O19" t="n">
+      <c r="R19" t="n">
         <v>77.82465815544128</v>
       </c>
-      <c r="R19" t="n">
+      <c r="U19" t="n">
         <v>70.55094838142395</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>71.40762805938721</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>70.30095756053925</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>70.45986354351044</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>70.54699063301086</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>70.52779197692871</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>74.83260035514832</v>
       </c>
     </row>
     <row r="20">
@@ -1504,33 +2241,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>-0.3534631651993525</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="n">
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="n">
         <v>-27.1827</v>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
         <v>71.80301547050476</v>
       </c>
-      <c r="L20" t="n">
+      <c r="O20" t="n">
         <v>67.43274033069611</v>
       </c>
-      <c r="O20" t="n">
+      <c r="R20" t="n">
         <v>78.36011350154877</v>
       </c>
-      <c r="R20" t="n">
+      <c r="U20" t="n">
         <v>73.10449182987213</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>71.36403024196625</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>71.4694082736969</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>71.67989313602448</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>70.35038769245148</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>72.30775356292725</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>75.17090290784836</v>
       </c>
     </row>
     <row r="21">
@@ -1557,33 +2327,66 @@
           <t>\</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
         <v>51.46190740116804</v>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="n">
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="n">
         <v>-150.8484</v>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
         <v>64.38460350036621</v>
       </c>
-      <c r="L21" t="n">
+      <c r="O21" t="n">
         <v>63.52652311325073</v>
       </c>
-      <c r="O21" t="n">
+      <c r="R21" t="n">
         <v>81.56867474317551</v>
       </c>
-      <c r="R21" t="n">
+      <c r="U21" t="n">
         <v>69.94550228118896</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>71.19808495044708</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>58.88660848140717</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>68.39650869369507</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>68.48113238811493</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>74.5064377784729</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>72.25974500179291</v>
       </c>
     </row>
     <row r="22">
@@ -1599,50 +2402,101 @@
         <v>71.7753</v>
       </c>
       <c r="D22" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="E22" s="5" t="n">
         <v>48.0013</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="F22" s="5" t="n">
         <v>2.9754</v>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G22" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="n">
         <v>54.6177</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="n">
+      <c r="J22" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="n">
         <v>109.2962</v>
       </c>
-      <c r="K22" t="n">
+      <c r="N22" t="n">
         <v>19.45809936523438</v>
       </c>
-      <c r="M22" t="n">
+      <c r="P22" t="n">
         <v>60.48505783081055</v>
       </c>
-      <c r="N22" t="n">
+      <c r="Q22" t="n">
         <v>50</v>
       </c>
-      <c r="P22" t="n">
+      <c r="S22" t="n">
         <v>-30.56501770019531</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="T22" t="n">
         <v>120</v>
       </c>
-      <c r="S22" t="n">
+      <c r="V22" t="n">
         <v>45.11756896972656</v>
       </c>
-      <c r="T22" t="n">
+      <c r="W22" t="n">
         <v>40</v>
       </c>
-      <c r="U22" t="n">
+      <c r="X22" t="n">
         <v>80</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>22.5233154296875</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>46.9628791809082</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>35</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>55.59963607788086</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>54.50478363037109</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>55.93772888183594</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>32.8129997253418</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>95</v>
+      </c>
+      <c r="AS22" t="n">
+        <v>46.17313766479492</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1658,47 +2512,96 @@
         <v>61.4115</v>
       </c>
       <c r="D23" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="E23" s="5" t="n">
         <v>145.4161</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="F23" s="5" t="n">
         <v>23.4426</v>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G23" s="5" t="n">
+        <v>295</v>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
         <v>242.8916</v>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="n">
+      <c r="J23" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="n">
         <v>485.663</v>
       </c>
-      <c r="K23" t="n">
+      <c r="M23" s="13" t="n"/>
+      <c r="N23" t="n">
         <v>161.4140014648438</v>
       </c>
-      <c r="M23" t="n">
+      <c r="P23" t="n">
         <v>174.9732666015625</v>
       </c>
-      <c r="N23" t="n">
+      <c r="Q23" t="n">
         <v>40</v>
       </c>
-      <c r="P23" t="n">
+      <c r="S23" t="n">
         <v>-4.313392639160156</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="T23" t="n">
         <v>335</v>
       </c>
-      <c r="S23" t="n">
+      <c r="V23" t="n">
         <v>113.0792236328125</v>
       </c>
-      <c r="T23" t="n">
+      <c r="W23" t="n">
         <v>30</v>
+      </c>
+      <c r="X23" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>107.4765777587891</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>50</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>155.5734252929688</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>35</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>161.0006256103516</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>35</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>165.6830749511719</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP23" t="n">
+        <v>114.0658111572266</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AS23" t="n">
+        <v>126.5128479003906</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1714,47 +2617,95 @@
         <v>67.60080000000001</v>
       </c>
       <c r="D24" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="E24" s="5" t="n">
         <v>48.2493</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="F24" s="5" t="n">
         <v>7.6203</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G24" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="n">
         <v>108.4434</v>
       </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="n">
+      <c r="J24" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="n">
         <v>219.0176</v>
       </c>
-      <c r="K24" t="n">
+      <c r="N24" t="n">
         <v>76.19950866699219</v>
       </c>
-      <c r="M24" t="n">
+      <c r="P24" t="n">
         <v>67.40234375</v>
       </c>
-      <c r="N24" t="n">
+      <c r="Q24" t="n">
         <v>25</v>
       </c>
-      <c r="P24" t="n">
+      <c r="S24" t="n">
         <v>5.866661071777344</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="T24" t="n">
         <v>135</v>
       </c>
-      <c r="S24" t="n">
+      <c r="V24" t="n">
         <v>68.044921875</v>
       </c>
-      <c r="T24" t="n">
+      <c r="W24" t="n">
         <v>25</v>
+      </c>
+      <c r="X24" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>51.16263580322266</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>40</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>73.37741851806641</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>25</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>76.03903961181641</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>25</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>80.8988037109375</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>30</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>58.30487823486328</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>85</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>56.8088264465332</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1770,48 +2721,96 @@
         <v>35.9121</v>
       </c>
       <c r="D25" s="5" t="n">
+        <v>305</v>
+      </c>
+      <c r="E25" s="5" t="n">
         <v>84.4406</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="F25" s="5" t="n">
         <v>0.0017869</v>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G25" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
         <v>142.739</v>
       </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="n">
+      <c r="J25" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="n">
         <v>284.9266</v>
       </c>
-      <c r="J25" s="10" t="n"/>
-      <c r="K25" t="n">
+      <c r="M25" s="10" t="n"/>
+      <c r="N25" t="n">
         <v>135.5852813720703</v>
       </c>
-      <c r="M25" t="n">
+      <c r="P25" t="n">
         <v>126.3647918701172</v>
       </c>
-      <c r="N25" t="n">
+      <c r="Q25" t="n">
         <v>60</v>
       </c>
-      <c r="P25" t="n">
+      <c r="S25" t="n">
         <v>-8.396797180175781</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="T25" t="n">
         <v>335</v>
       </c>
-      <c r="S25" t="n">
+      <c r="V25" t="n">
         <v>101.8771743774414</v>
       </c>
-      <c r="T25" t="n">
+      <c r="W25" t="n">
         <v>60</v>
+      </c>
+      <c r="X25" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>105.4740600585938</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>40</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>137.1975402832031</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>40</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>135.3927307128906</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>40</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>133.8984832763672</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>45</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>149.968017578125</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>105</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>76.27444458007812</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="26">
@@ -1827,46 +2826,94 @@
         <v>79.6031</v>
       </c>
       <c r="D26" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="E26" s="5" t="n">
         <v>112.8086</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="F26" s="5" t="n">
         <v>6.5136</v>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G26" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="n">
         <v>127.3407</v>
       </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="n">
+      <c r="J26" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="n">
         <v>253.7063</v>
       </c>
-      <c r="K26" t="n">
+      <c r="N26" t="n">
         <v>122.4537963867188</v>
       </c>
-      <c r="M26" t="n">
+      <c r="P26" t="n">
         <v>151.0030059814453</v>
       </c>
-      <c r="N26" t="n">
+      <c r="Q26" t="n">
         <v>35</v>
       </c>
-      <c r="P26" t="n">
+      <c r="S26" t="n">
         <v>97.13450622558594</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="T26" t="n">
         <v>70</v>
       </c>
-      <c r="S26" t="n">
+      <c r="V26" t="n">
         <v>127.6560440063477</v>
       </c>
-      <c r="T26" t="n">
+      <c r="W26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" t="n">
+        <v>65</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>110.8215637207031</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>65</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>121.8299026489258</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>65</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>122.6051483154297</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>65</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>200.9173889160156</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>168.0099182128906</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>117.6930541992188</v>
+      </c>
+      <c r="AT26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1883,47 +2930,95 @@
         <v>79.5839</v>
       </c>
       <c r="D27" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="E27" s="5" t="n">
         <v>56.0085</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="F27" s="5" t="n">
         <v>42.9352</v>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G27" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
         <v>63.4823</v>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="n">
+      <c r="J27" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="n">
         <v>127.2308</v>
       </c>
-      <c r="K27" t="n">
+      <c r="N27" t="n">
         <v>95.11552429199219</v>
       </c>
-      <c r="M27" t="n">
+      <c r="P27" t="n">
         <v>84.47927856445312</v>
       </c>
-      <c r="N27" t="n">
+      <c r="Q27" t="n">
         <v>40</v>
       </c>
-      <c r="P27" t="n">
+      <c r="S27" t="n">
         <v>15.19478607177734</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="T27" t="n">
         <v>215</v>
       </c>
-      <c r="S27" t="n">
+      <c r="V27" t="n">
         <v>92.37336730957031</v>
       </c>
-      <c r="T27" t="n">
+      <c r="W27" t="n">
         <v>40</v>
+      </c>
+      <c r="X27" t="n">
+        <v>45</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>79.63713073730469</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>55</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>91.26934814453125</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>40</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>95.80051422119141</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>45</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>94.17977905273438</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>45</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>80.13362121582031</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>130</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>60.47091293334961</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1939,41 +3034,89 @@
         <v>76.46120000000001</v>
       </c>
       <c r="D28" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="E28" s="5" t="n">
         <v>87.8904</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="F28" s="5" t="n">
         <v>38.1008</v>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G28" s="5" t="n">
+        <v>235</v>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="n">
         <v>92.0838</v>
       </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="n">
+      <c r="J28" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="n">
         <v>184.2133</v>
       </c>
-      <c r="K28" t="n">
+      <c r="N28" t="n">
         <v>146.6000366210938</v>
       </c>
-      <c r="M28" t="n">
+      <c r="P28" t="n">
         <v>116.0833129882812</v>
       </c>
-      <c r="N28" t="n">
+      <c r="Q28" t="n">
         <v>60</v>
       </c>
-      <c r="P28" t="n">
+      <c r="S28" t="n">
         <v>19.94272613525391</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="T28" t="n">
         <v>120</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>127.320915222168</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>60</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>143.0389709472656</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>147.1386566162109</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>134.2376403808594</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>60</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>157.8865966796875</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>59.74942016601562</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1989,47 +3132,95 @@
         <v>57.2864</v>
       </c>
       <c r="D29" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="E29" s="5" t="n">
         <v>74.7406</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="F29" s="5" t="n">
         <v>20.1644</v>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G29" s="5" t="n">
+        <v>215</v>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
         <v>92.71129999999999</v>
       </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="n">
+      <c r="J29" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="n">
         <v>185.4194</v>
       </c>
-      <c r="K29" t="n">
+      <c r="N29" t="n">
         <v>99.73930358886719</v>
       </c>
-      <c r="M29" t="n">
+      <c r="P29" t="n">
         <v>89.82148742675781</v>
       </c>
-      <c r="N29" t="n">
+      <c r="Q29" t="n">
         <v>45</v>
       </c>
-      <c r="P29" t="n">
+      <c r="S29" t="n">
         <v>41.55772399902344</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="T29" t="n">
         <v>65</v>
       </c>
-      <c r="S29" t="n">
+      <c r="V29" t="n">
         <v>97.54011535644531</v>
       </c>
-      <c r="T29" t="n">
+      <c r="W29" t="n">
         <v>50</v>
+      </c>
+      <c r="X29" t="n">
+        <v>50</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>94.68830871582031</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>50</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>97.5943603515625</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>98.70677185058594</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>50</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>101.621696472168</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>60</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>98.64247131347656</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>66.50881958007812</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2045,47 +3236,95 @@
         <v>60.2236</v>
       </c>
       <c r="D30" s="5" t="n">
+        <v>240</v>
+      </c>
+      <c r="E30" s="5" t="n">
         <v>85.47369999999999</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="F30" s="5" t="n">
         <v>2.9808</v>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G30" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="n">
         <v>91.10380000000001</v>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="n">
+      <c r="J30" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="n">
         <v>181.5097</v>
       </c>
-      <c r="K30" t="n">
+      <c r="N30" t="n">
         <v>109.523681640625</v>
       </c>
-      <c r="M30" t="n">
+      <c r="P30" t="n">
         <v>112.8166275024414</v>
       </c>
-      <c r="N30" t="n">
+      <c r="Q30" t="n">
         <v>50</v>
       </c>
-      <c r="P30" t="n">
+      <c r="S30" t="n">
         <v>39.81376647949219</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="T30" t="n">
         <v>340</v>
       </c>
-      <c r="S30" t="n">
+      <c r="V30" t="n">
         <v>91.2020263671875</v>
       </c>
-      <c r="T30" t="n">
+      <c r="W30" t="n">
         <v>60</v>
+      </c>
+      <c r="X30" t="n">
+        <v>55</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>83.79324340820312</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>55</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>109.4817810058594</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>55</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>109.7333526611328</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>55</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>110.1037979125977</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>50</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>110.9524688720703</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>105</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>79.58257293701172</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -2101,47 +3340,95 @@
         <v>74.75539999999999</v>
       </c>
       <c r="D31" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="E31" s="5" t="n">
         <v>86.6242</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="F31" s="5" t="n">
         <v>36.8083</v>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G31" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
         <v>128.3617</v>
       </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="n">
+      <c r="J31" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="n">
         <v>256.5043</v>
       </c>
-      <c r="K31" t="n">
+      <c r="N31" t="n">
         <v>116.7160568237305</v>
       </c>
-      <c r="M31" t="n">
+      <c r="P31" t="n">
         <v>105.5226974487305</v>
       </c>
-      <c r="N31" t="n">
+      <c r="Q31" t="n">
         <v>40</v>
       </c>
-      <c r="P31" t="n">
+      <c r="S31" t="n">
         <v>23.30689239501953</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="T31" t="n">
         <v>225</v>
       </c>
-      <c r="S31" t="n">
+      <c r="V31" t="n">
         <v>94.0443115234375</v>
       </c>
-      <c r="T31" t="n">
+      <c r="W31" t="n">
         <v>40</v>
+      </c>
+      <c r="X31" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>64.1058349609375</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>55</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>112.9663696289062</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>40</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>117.8259887695312</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>40</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>210.3694763183594</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>85.7930908203125</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>95</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>91.78579711914062</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2156,19 +3443,17 @@
       <c r="C32" s="9" t="n">
         <v>279.5702</v>
       </c>
-      <c r="D32" s="5" t="n">
+      <c r="D32" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="E32" s="5" t="n">
         <v>163.1491</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="F32" s="5" t="n">
         <v>128.2192855461584</v>
       </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G32" s="5" t="n">
-        <v>154.6361</v>
+        <v>115</v>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
@@ -2178,29 +3463,76 @@
       <c r="I32" s="5" t="n">
         <v>154.6361</v>
       </c>
-      <c r="K32" t="n">
+      <c r="J32" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>154.6361</v>
+      </c>
+      <c r="N32" t="n">
         <v>197.8385772705078</v>
       </c>
-      <c r="M32" t="n">
+      <c r="P32" t="n">
         <v>285.4031982421875</v>
       </c>
-      <c r="N32" t="n">
+      <c r="Q32" t="n">
         <v>115</v>
       </c>
-      <c r="P32" t="n">
+      <c r="S32" t="n">
         <v>181.1156005859375</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>120</v>
-      </c>
-      <c r="S32" t="n">
-        <v>265.1717834472656</v>
       </c>
       <c r="T32" t="n">
         <v>120</v>
       </c>
-      <c r="U32" t="n">
+      <c r="V32" t="n">
+        <v>265.1717834472656</v>
+      </c>
+      <c r="W32" t="n">
+        <v>120</v>
+      </c>
+      <c r="X32" t="n">
         <v>130</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>261.6098937988281</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>115</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>297.2069702148438</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>120</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>295.4985961914062</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>115</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>298.315185546875</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>120</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>230.3070983886719</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>135</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>243.1541137695312</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="33">
@@ -2215,19 +3547,17 @@
       <c r="C33" s="9" t="n">
         <v>220.9999</v>
       </c>
-      <c r="D33" s="5" t="n">
+      <c r="D33" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="E33" s="5" t="n">
         <v>243.268</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="F33" s="5" t="n">
         <v>46.07324551248713</v>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G33" s="5" t="n">
-        <v>153.9843</v>
+        <v>245</v>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
@@ -2237,26 +3567,76 @@
       <c r="I33" s="5" t="n">
         <v>153.9843</v>
       </c>
-      <c r="K33" t="n">
+      <c r="J33" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>153.9843</v>
+      </c>
+      <c r="N33" t="n">
         <v>296.5382690429688</v>
       </c>
-      <c r="M33" t="n">
+      <c r="P33" t="n">
         <v>323.2284545898438</v>
       </c>
-      <c r="N33" t="n">
+      <c r="Q33" t="n">
         <v>135</v>
       </c>
-      <c r="P33" t="n">
+      <c r="S33" t="n">
         <v>101.2586517333984</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="T33" t="n">
         <v>145</v>
       </c>
-      <c r="S33" t="n">
+      <c r="V33" t="n">
         <v>251.2278137207031</v>
       </c>
-      <c r="T33" t="n">
+      <c r="W33" t="n">
         <v>140</v>
+      </c>
+      <c r="X33" t="n">
+        <v>135</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>254.0560455322266</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>150</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>300.412353515625</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>135</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>302.0830993652344</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>135</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>298.1703491210938</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>135</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>250.2373962402344</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>175</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>218.351318359375</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>115</v>
       </c>
     </row>
     <row r="34">
@@ -2271,19 +3651,17 @@
       <c r="C34" s="9" t="n">
         <v>186.3073</v>
       </c>
-      <c r="D34" s="5" t="n">
+      <c r="D34" s="9" t="n">
+        <v>245</v>
+      </c>
+      <c r="E34" s="5" t="n">
         <v>243.268</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="F34" s="5" t="n">
         <v>56.37320603333124</v>
       </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G34" s="5" t="n">
-        <v>154.1875</v>
+        <v>90</v>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
@@ -2293,26 +3671,76 @@
       <c r="I34" s="5" t="n">
         <v>154.1875</v>
       </c>
-      <c r="K34" t="n">
+      <c r="J34" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>154.1875</v>
+      </c>
+      <c r="N34" t="n">
         <v>230.4547119140625</v>
       </c>
-      <c r="M34" t="n">
+      <c r="P34" t="n">
         <v>220.6366271972656</v>
       </c>
-      <c r="N34" t="n">
+      <c r="Q34" t="n">
         <v>130</v>
       </c>
-      <c r="P34" t="n">
+      <c r="S34" t="n">
         <v>91.90601348876953</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="T34" t="n">
         <v>135</v>
       </c>
-      <c r="S34" t="n">
+      <c r="V34" t="n">
         <v>226.6964416503906</v>
       </c>
-      <c r="T34" t="n">
+      <c r="W34" t="n">
         <v>130</v>
+      </c>
+      <c r="X34" t="n">
+        <v>130</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>195.5531463623047</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>125</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>241.3056793212891</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>130</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>230.6870880126953</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>130</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>243.4823608398438</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>130</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>193.0436096191406</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>150</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>205.3022003173828</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -2327,19 +3755,17 @@
       <c r="C35" s="9" t="n">
         <v>155.2635</v>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D35" s="9" t="n">
+        <v>275</v>
+      </c>
+      <c r="E35" s="5" t="n">
         <v>243.268</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="F35" s="5" t="n">
         <v>0.5995429438134749</v>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G35" s="5" t="n">
-        <v>153.5179</v>
+        <v>105</v>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
@@ -2349,26 +3775,76 @@
       <c r="I35" s="5" t="n">
         <v>153.5179</v>
       </c>
-      <c r="K35" t="n">
+      <c r="J35" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>153.5179</v>
+      </c>
+      <c r="N35" t="n">
         <v>244.2931823730469</v>
       </c>
-      <c r="M35" t="n">
+      <c r="P35" t="n">
         <v>245.7116088867188</v>
       </c>
-      <c r="N35" t="n">
+      <c r="Q35" t="n">
         <v>200</v>
       </c>
-      <c r="P35" t="n">
+      <c r="S35" t="n">
         <v>62.16912078857422</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="T35" t="n">
         <v>190</v>
       </c>
-      <c r="S35" t="n">
+      <c r="V35" t="n">
         <v>225.9434967041016</v>
       </c>
-      <c r="T35" t="n">
+      <c r="W35" t="n">
         <v>200</v>
+      </c>
+      <c r="X35" t="n">
+        <v>205</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>217.9620666503906</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>200</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>244.22265625</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>200</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>240.4562683105469</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>205</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>245.5692443847656</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>200</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>230.5582122802734</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>225</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>172.430419921875</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>165</v>
       </c>
     </row>
     <row r="36">
@@ -2383,19 +3859,17 @@
       <c r="C36" s="9" t="n">
         <v>192.7964</v>
       </c>
-      <c r="D36" s="5" t="n">
+      <c r="D36" s="9" t="n">
+        <v>275</v>
+      </c>
+      <c r="E36" s="5" t="n">
         <v>163.1491</v>
       </c>
-      <c r="E36" s="5" t="n">
+      <c r="F36" s="5" t="n">
         <v>67.71863377151476</v>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G36" s="5" t="n">
-        <v>153.5087</v>
+        <v>70</v>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
@@ -2405,26 +3879,76 @@
       <c r="I36" s="5" t="n">
         <v>153.5087</v>
       </c>
-      <c r="K36" t="n">
+      <c r="J36" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="n">
+        <v>153.5087</v>
+      </c>
+      <c r="N36" t="n">
         <v>213.9585418701172</v>
       </c>
-      <c r="M36" t="n">
+      <c r="P36" t="n">
         <v>213.0440368652344</v>
       </c>
-      <c r="N36" t="n">
+      <c r="Q36" t="n">
         <v>90</v>
       </c>
-      <c r="P36" t="n">
+      <c r="S36" t="n">
         <v>149.1197052001953</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="T36" t="n">
         <v>95</v>
       </c>
-      <c r="S36" t="n">
+      <c r="V36" t="n">
         <v>214.0133972167969</v>
       </c>
-      <c r="T36" t="n">
+      <c r="W36" t="n">
         <v>90</v>
+      </c>
+      <c r="X36" t="n">
+        <v>90</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>213.7317810058594</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>90</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>215.2785797119141</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>90</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>210.7884826660156</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM36" t="n">
+        <v>215.46875</v>
+      </c>
+      <c r="AN36" t="n">
+        <v>90</v>
+      </c>
+      <c r="AP36" t="n">
+        <v>193.5937194824219</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>95</v>
+      </c>
+      <c r="AS36" t="n">
+        <v>194.0391082763672</v>
+      </c>
+      <c r="AT36" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="37">
@@ -2439,19 +3963,17 @@
       <c r="C37" s="9" t="n">
         <v>212.5705</v>
       </c>
-      <c r="D37" s="5" t="n">
+      <c r="D37" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="E37" s="5" t="n">
         <v>163.1491</v>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="F37" s="5" t="n">
         <v>104.8694093902491</v>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G37" s="5" t="n">
-        <v>153.8387</v>
+        <v>195</v>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
@@ -2461,26 +3983,76 @@
       <c r="I37" s="5" t="n">
         <v>153.8387</v>
       </c>
-      <c r="K37" t="n">
+      <c r="J37" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="n">
+        <v>153.8387</v>
+      </c>
+      <c r="N37" t="n">
         <v>181.1307220458984</v>
       </c>
-      <c r="M37" t="n">
+      <c r="P37" t="n">
         <v>186.1939697265625</v>
       </c>
-      <c r="N37" t="n">
+      <c r="Q37" t="n">
         <v>145</v>
       </c>
-      <c r="P37" t="n">
+      <c r="S37" t="n">
         <v>105.5374603271484</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="T37" t="n">
         <v>165</v>
       </c>
-      <c r="S37" t="n">
+      <c r="V37" t="n">
         <v>179.5286407470703</v>
       </c>
-      <c r="T37" t="n">
+      <c r="W37" t="n">
         <v>145</v>
+      </c>
+      <c r="X37" t="n">
+        <v>150</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>177.2041625976562</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>145</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>180.8521423339844</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>145</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>179.6074523925781</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>150</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>184.5145568847656</v>
+      </c>
+      <c r="AN37" t="n">
+        <v>145</v>
+      </c>
+      <c r="AP37" t="n">
+        <v>180.3097991943359</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>155</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>156.7861633300781</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>135</v>
       </c>
     </row>
     <row r="38">
@@ -2495,19 +4067,17 @@
       <c r="C38" s="9" t="n">
         <v>190.4762</v>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="D38" s="9" t="n">
+        <v>195</v>
+      </c>
+      <c r="E38" s="5" t="n">
         <v>163.1491</v>
       </c>
-      <c r="E38" s="5" t="n">
+      <c r="F38" s="5" t="n">
         <v>62.3767240626488</v>
       </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G38" s="5" t="n">
-        <v>153.9645</v>
+        <v>240</v>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
@@ -2517,20 +4087,70 @@
       <c r="I38" s="5" t="n">
         <v>153.9645</v>
       </c>
-      <c r="K38" t="n">
+      <c r="J38" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>153.9645</v>
+      </c>
+      <c r="N38" t="n">
         <v>267.6002197265625</v>
       </c>
-      <c r="M38" t="n">
+      <c r="P38" t="n">
         <v>278.4971313476562</v>
       </c>
-      <c r="N38" t="n">
+      <c r="Q38" t="n">
         <v>130</v>
       </c>
-      <c r="P38" t="n">
+      <c r="S38" t="n">
         <v>138.6098327636719</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="T38" t="n">
         <v>120</v>
+      </c>
+      <c r="X38" t="n">
+        <v>130</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>258.2368774414062</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>271.3315734863281</v>
+      </c>
+      <c r="AH38" t="n">
+        <v>130</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>272.2751159667969</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>135</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>273.451904296875</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>135</v>
+      </c>
+      <c r="AP38" t="n">
+        <v>262.7337036132812</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>135</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>222.6571044921875</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>110</v>
       </c>
     </row>
     <row r="39">
@@ -2545,19 +4165,17 @@
       <c r="C39" s="9" t="n">
         <v>198.5261</v>
       </c>
-      <c r="D39" s="5" t="n">
+      <c r="D39" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="E39" s="5" t="n">
         <v>210.4307</v>
       </c>
-      <c r="E39" s="5" t="n">
+      <c r="F39" s="5" t="n">
         <v>84.94764448236532</v>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G39" s="5" t="n">
-        <v>153.8718</v>
+        <v>155</v>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
@@ -2567,26 +4185,76 @@
       <c r="I39" s="5" t="n">
         <v>153.8718</v>
       </c>
-      <c r="K39" t="n">
+      <c r="J39" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>153.8718</v>
+      </c>
+      <c r="N39" t="n">
         <v>281.9173583984375</v>
       </c>
-      <c r="M39" t="n">
+      <c r="P39" t="n">
         <v>297.396728515625</v>
-      </c>
-      <c r="N39" t="n">
-        <v>125</v>
-      </c>
-      <c r="P39" t="n">
-        <v>216.1502990722656</v>
       </c>
       <c r="Q39" t="n">
         <v>125</v>
       </c>
       <c r="S39" t="n">
-        <v>281.90380859375</v>
+        <v>216.1502990722656</v>
       </c>
       <c r="T39" t="n">
         <v>125</v>
+      </c>
+      <c r="V39" t="n">
+        <v>281.90380859375</v>
+      </c>
+      <c r="W39" t="n">
+        <v>125</v>
+      </c>
+      <c r="X39" t="n">
+        <v>125</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>275.417724609375</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>125</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>284.4364624023438</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>125</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>284.7573547363281</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>125</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>281.7852172851562</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>125</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>272.2428894042969</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>130</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>227.6891479492188</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="40">
@@ -2601,19 +4269,17 @@
       <c r="C40" s="9" t="n">
         <v>188.0244</v>
       </c>
-      <c r="D40" s="5" t="n">
+      <c r="D40" s="9" t="n">
+        <v>215</v>
+      </c>
+      <c r="E40" s="5" t="n">
         <v>163.1491</v>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="F40" s="5" t="n">
         <v>73.87837727987502</v>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G40" s="5" t="n">
-        <v>153.6361</v>
+        <v>100</v>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
@@ -2623,26 +4289,76 @@
       <c r="I40" s="5" t="n">
         <v>153.6361</v>
       </c>
-      <c r="K40" t="n">
+      <c r="J40" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>153.6361</v>
+      </c>
+      <c r="N40" t="n">
         <v>227.6520690917969</v>
       </c>
-      <c r="M40" t="n">
+      <c r="P40" t="n">
         <v>238.9959716796875</v>
       </c>
-      <c r="N40" t="n">
+      <c r="Q40" t="n">
         <v>130</v>
       </c>
-      <c r="P40" t="n">
+      <c r="S40" t="n">
         <v>142.0441284179688</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="T40" t="n">
         <v>125</v>
       </c>
-      <c r="S40" t="n">
+      <c r="V40" t="n">
         <v>220.6580505371094</v>
       </c>
-      <c r="T40" t="n">
+      <c r="W40" t="n">
         <v>130</v>
+      </c>
+      <c r="X40" t="n">
+        <v>135</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>218.357177734375</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>135</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>225.7833404541016</v>
+      </c>
+      <c r="AH40" t="n">
+        <v>135</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>228.4818572998047</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>135</v>
+      </c>
+      <c r="AM40" t="n">
+        <v>224.0914306640625</v>
+      </c>
+      <c r="AN40" t="n">
+        <v>130</v>
+      </c>
+      <c r="AP40" t="n">
+        <v>202.5383911132812</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>145</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>190.1109313964844</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="41">
@@ -2657,19 +4373,17 @@
       <c r="C41" s="9" t="n">
         <v>197.3272</v>
       </c>
-      <c r="D41" s="5" t="n">
+      <c r="D41" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="E41" s="5" t="n">
         <v>243.268</v>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="F41" s="5" t="n">
         <v>95.83648987338964</v>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>\</t>
-        </is>
-      </c>
       <c r="G41" s="5" t="n">
-        <v>153.791</v>
+        <v>190</v>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
@@ -2679,26 +4393,76 @@
       <c r="I41" s="5" t="n">
         <v>153.791</v>
       </c>
-      <c r="K41" t="n">
+      <c r="J41" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>\</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>153.791</v>
+      </c>
+      <c r="N41" t="n">
         <v>224.6213073730469</v>
       </c>
-      <c r="M41" t="n">
+      <c r="P41" t="n">
         <v>224.9940185546875</v>
       </c>
-      <c r="N41" t="n">
+      <c r="Q41" t="n">
         <v>140</v>
       </c>
-      <c r="P41" t="n">
+      <c r="S41" t="n">
         <v>98.53268432617188</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="T41" t="n">
         <v>150</v>
       </c>
-      <c r="S41" t="n">
+      <c r="V41" t="n">
         <v>210.8045654296875</v>
       </c>
-      <c r="T41" t="n">
+      <c r="W41" t="n">
         <v>145</v>
+      </c>
+      <c r="X41" t="n">
+        <v>145</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>195.6446533203125</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>145</v>
+      </c>
+      <c r="AG41" t="n">
+        <v>225.4454803466797</v>
+      </c>
+      <c r="AH41" t="n">
+        <v>145</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>222.0240936279297</v>
+      </c>
+      <c r="AK41" t="n">
+        <v>145</v>
+      </c>
+      <c r="AM41" t="n">
+        <v>222.0058288574219</v>
+      </c>
+      <c r="AN41" t="n">
+        <v>145</v>
+      </c>
+      <c r="AP41" t="n">
+        <v>200.0965881347656</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>160</v>
+      </c>
+      <c r="AS41" t="n">
+        <v>174.3958129882812</v>
+      </c>
+      <c r="AT41" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1"/>
@@ -2727,7 +4491,10 @@
       <c r="E62" s="6" t="n"/>
       <c r="F62" s="6" t="n"/>
       <c r="G62" s="6" t="n"/>
-      <c r="I62" s="12" t="n"/>
+      <c r="H62" s="6" t="n"/>
+      <c r="I62" s="6" t="n"/>
+      <c r="J62" s="6" t="n"/>
+      <c r="L62" s="12" t="n"/>
     </row>
     <row r="63" ht="14.25" customHeight="1"/>
     <row r="64" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
strategy 2 promising now with SSM
</commit_message>
<xml_diff>
--- a/results_v3.xlsx
+++ b/results_v3.xlsx
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>69.08353269100189</v>
+        <v>50.01786351203918</v>
       </c>
       <c r="O2" t="n">
         <v>66.20668023824692</v>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>66.37006998062134</v>
+        <v>49.07691180706024</v>
       </c>
       <c r="O8" t="n">
         <v>66.68574512004852</v>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>66.06106162071228</v>
+        <v>-0.1446962356567383</v>
       </c>
       <c r="O12" t="n">
         <v>56.76135122776031</v>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>63.18274736404419</v>
+        <v>43.63647103309631</v>
       </c>
       <c r="O18" t="n">
         <v>66.30968749523163</v>
@@ -2433,7 +2433,7 @@
         <v>109.2962</v>
       </c>
       <c r="N22" t="n">
-        <v>19.45809936523438</v>
+        <v>45.04288101196289</v>
       </c>
       <c r="P22" t="n">
         <v>60.48505783081055</v>
@@ -2454,7 +2454,7 @@
         <v>40</v>
       </c>
       <c r="X22" t="n">
-        <v>80</v>
+        <v>275</v>
       </c>
       <c r="AA22" t="n">
         <v>22.5233154296875</v>
@@ -3065,7 +3065,7 @@
         <v>184.2133</v>
       </c>
       <c r="N28" t="n">
-        <v>146.6000366210938</v>
+        <v>121.4229583740234</v>
       </c>
       <c r="P28" t="n">
         <v>116.0833129882812</v>
@@ -3080,7 +3080,7 @@
         <v>120</v>
       </c>
       <c r="X28" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD28" t="n">
         <v>127.320915222168</v>
@@ -3475,7 +3475,7 @@
         <v>154.6361</v>
       </c>
       <c r="N32" t="n">
-        <v>197.8385772705078</v>
+        <v>122.9351806640625</v>
       </c>
       <c r="P32" t="n">
         <v>285.4031982421875</v>
@@ -3496,7 +3496,7 @@
         <v>120</v>
       </c>
       <c r="X32" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="AD32" t="n">
         <v>261.6098937988281</v>
@@ -4099,7 +4099,7 @@
         <v>153.9645</v>
       </c>
       <c r="N38" t="n">
-        <v>267.6002197265625</v>
+        <v>268.207763671875</v>
       </c>
       <c r="P38" t="n">
         <v>278.4971313476562</v>

</xml_diff>